<commit_message>
Case study pictures from Higgsfield: the module, its test, and the Andheri set
api/cms/_images.js submits a slot's prompt in the house style to
Higgsfield's API (Key id:secret, submit then poll the status URL, per
docs.higgsfield.ai), waits for the picture and copies it into our own
storage under the case's slug. scripts/images.test.js runs that path
against a stand-in API: a slow job, a refused one, a bad key, no key.

The nine Andheri illustrations were generated once through the Higgsfield
MCP with the same prompts and style and are referenced from the example
workbook, so /casestudy/ shows the finished design.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016g4QfvH4SYnh6fLzsEaQQF
</commit_message>
<xml_diff>
--- a/examples/andheri-case.xlsx
+++ b/examples/andheri-case.xlsx
@@ -348,7 +348,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1522" uniqueCount="746">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1540" uniqueCount="756">
   <si>
     <t>Building a case study</t>
   </si>
@@ -2569,28 +2569,58 @@
     <t>Two modern office buildings in a Mumbai suburb at dusk, one finished glass tower and one under construction with cranes, an elevated metro line in the foreground, monsoon sky clearing</t>
   </si>
   <si>
+    <t>https://d8j0ntlcm91z4.cloudfront.net/user_3Fo7i4SvZozV6ke0Djuea827rgj/hf_20261021_224738_f96800db-c373-43a1-a4c0-86d8f52425e4.png</t>
+  </si>
+  <si>
+    <t>AI-generated illustration (Higgsfield)</t>
+  </si>
+  <si>
     <t>An empty bare-shell office floor with floor-to-ceiling windows looking out over Andheri East, late afternoon light, measuring tape and floor plans on the concrete floor</t>
   </si>
   <si>
+    <t>https://d8j0ntlcm91z4.cloudfront.net/user_3Fo7i4SvZozV6ke0Djuea827rgj/hf_20261021_224708_79f674bd-40a9-415e-8d52-7d163c3a9c73.png</t>
+  </si>
+  <si>
     <t>A new office tower beside an elevated metro station at street level, people walking from the station entrance, Mumbai, early morning</t>
   </si>
   <si>
+    <t>https://d8j0ntlcm91z4.cloudfront.net/user_3Fo7i4SvZozV6ke0Djuea827rgj/hf_20261021_224709_a33c27ba-bf66-4ad9-8c9f-8ae60d64dd8c.png</t>
+  </si>
+  <si>
     <t>A busy Mumbai business district street with Grade A office towers, taxis and office workers, overcast bright sky</t>
   </si>
   <si>
+    <t>https://d8j0ntlcm91z4.cloudfront.net/user_3Fo7i4SvZozV6ke0Djuea827rgj/hf_20261021_224709_74e781c3-32bb-4c56-ba29-2ab581eb25a3.png</t>
+  </si>
+  <si>
     <t>An elevated metro viaduct curving past office towers towards an airport terminal, aircraft landing in the distance, Mumbai</t>
   </si>
   <si>
+    <t>https://d8j0ntlcm91z4.cloudfront.net/user_3Fo7i4SvZozV6ke0Djuea827rgj/hf_20261021_224737_72e23284-41af-44f6-bdbe-2c9848c8c719.png</t>
+  </si>
+  <si>
     <t>A managed office interior with a client meeting in a glass cabin, city view of Andheri East through the window</t>
   </si>
   <si>
+    <t>https://d8j0ntlcm91z4.cloudfront.net/user_3Fo7i4SvZozV6ke0Djuea827rgj/hf_20261021_224708_cf24c231-cc12-4b8c-b9cf-7113f26ed66b.png</t>
+  </si>
+  <si>
     <t>A broker showing an office floor to two clients, floor plan in hand, large windows, Mumbai skyline</t>
   </si>
   <si>
+    <t>https://d8j0ntlcm91z4.cloudfront.net/user_3Fo7i4SvZozV6ke0Djuea827rgj/hf_20261021_224737_62e955e1-1914-4ff2-9cab-320ba490c692.png</t>
+  </si>
+  <si>
     <t>A row of coworking centre signs along a busy Andheri Kurla Road, evening, neon and glass</t>
   </si>
   <si>
+    <t>https://d8j0ntlcm91z4.cloudfront.net/user_3Fo7i4SvZozV6ke0Djuea827rgj/hf_20261021_224753_06320c03-f620-4731-9cd8-c743827c8b5d.png</t>
+  </si>
+  <si>
     <t>Aerial view of Marol at dusk, two metro lines crossing, the airport runway lights beyond</t>
+  </si>
+  <si>
+    <t>https://d8j0ntlcm91z4.cloudfront.net/user_3Fo7i4SvZozV6ke0Djuea827rgj/hf_20261021_224737_55db2f1f-9306-438b-996f-a7585c1fdb2e.png</t>
   </si>
 </sst>
 </file>
@@ -8849,76 +8879,130 @@
     <row r="398" spans="1:1" x14ac:dyDescent="0.25"/>
     <row r="399" spans="1:1" x14ac:dyDescent="0.25"/>
     <row r="400" spans="1:1" x14ac:dyDescent="0.25"/>
-    <row r="401" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
         <v>332</v>
       </c>
       <c r="B401" t="s">
         <v>737</v>
       </c>
-    </row>
-    <row r="402" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C401" t="s">
+        <v>738</v>
+      </c>
+      <c r="D401" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="402" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
         <v>342</v>
       </c>
       <c r="B402" t="s">
-        <v>738</v>
-      </c>
-    </row>
-    <row r="403" spans="1:2" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+      <c r="C402" t="s">
+        <v>741</v>
+      </c>
+      <c r="D402" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="403" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
         <v>346</v>
       </c>
       <c r="B403" t="s">
+        <v>742</v>
+      </c>
+      <c r="C403" t="s">
+        <v>743</v>
+      </c>
+      <c r="D403" t="s">
         <v>739</v>
       </c>
     </row>
-    <row r="404" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
         <v>353</v>
       </c>
       <c r="B404" t="s">
-        <v>740</v>
-      </c>
-    </row>
-    <row r="405" spans="1:2" x14ac:dyDescent="0.25">
+        <v>744</v>
+      </c>
+      <c r="C404" t="s">
+        <v>745</v>
+      </c>
+      <c r="D404" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="405" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
         <v>360</v>
       </c>
       <c r="B405" t="s">
-        <v>741</v>
-      </c>
-    </row>
-    <row r="406" spans="1:2" x14ac:dyDescent="0.25">
+        <v>746</v>
+      </c>
+      <c r="C405" t="s">
+        <v>747</v>
+      </c>
+      <c r="D405" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="406" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
         <v>363</v>
       </c>
       <c r="B406" t="s">
-        <v>742</v>
-      </c>
-    </row>
-    <row r="407" spans="1:2" x14ac:dyDescent="0.25">
+        <v>748</v>
+      </c>
+      <c r="C406" t="s">
+        <v>749</v>
+      </c>
+      <c r="D406" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="407" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
         <v>548</v>
       </c>
       <c r="B407" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="408" spans="1:2" x14ac:dyDescent="0.25">
+        <v>750</v>
+      </c>
+      <c r="C407" t="s">
+        <v>751</v>
+      </c>
+      <c r="D407" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="408" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
         <v>366</v>
       </c>
       <c r="B408" t="s">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="409" spans="1:2" x14ac:dyDescent="0.25">
+        <v>752</v>
+      </c>
+      <c r="C408" t="s">
+        <v>753</v>
+      </c>
+      <c r="D408" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="409" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
         <v>372</v>
       </c>
       <c r="B409" t="s">
-        <v>745</v>
+        <v>754</v>
+      </c>
+      <c r="C409" t="s">
+        <v>755</v>
+      </c>
+      <c r="D409" t="s">
+        <v>739</v>
       </c>
     </row>
   </sheetData>

</xml_diff>